<commit_message>
added a new script
</commit_message>
<xml_diff>
--- a/myPortfolioManagement/MeteoraGlobalEquityFund/Data/stock_screening.xlsx
+++ b/myPortfolioManagement/MeteoraGlobalEquityFund/Data/stock_screening.xlsx
@@ -1064,12 +1064,11 @@
   <cols>
     <col bestFit="1" min="1" max="1" width="11.140625"/>
     <col bestFit="1" min="2" max="2" width="28.140625"/>
-    <col bestFit="1" min="3" max="3" width="21.7109375"/>
-    <col bestFit="1" min="4" max="4" width="33.8515625"/>
-    <col customWidth="1" min="5" max="5" width="8.140625"/>
-    <col bestFit="1" min="6" max="6" width="10.140625"/>
+    <col customWidth="1" hidden="1" min="3" max="4" width="0"/>
+    <col customWidth="1" hidden="1" min="5" max="5" width="8.140625"/>
+    <col customWidth="1" hidden="1" min="6" max="6" width="0"/>
     <col bestFit="1" min="7" max="7" width="14.7109375"/>
-    <col bestFit="1" min="8" max="8" width="11.421875"/>
+    <col customWidth="1" hidden="1" min="8" max="8" width="0"/>
   </cols>
   <sheetData>
     <row r="1" ht="14.25">
@@ -3418,7 +3417,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="containsText" priority="1" id="{00F30013-00A8-4DA3-937D-002A0003001D}">
+          <x14:cfRule type="containsText" priority="1" id="{0000001B-0041-429A-9D6E-00AC007E009C}">
             <xm:f>NOT(ISERROR(SEARCH("$J$5",I2)))</xm:f>
             <xm:f>$J$5</xm:f>
             <x14:dxf>
@@ -5408,7 +5407,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="10" operator="lessThan" id="{00FB001B-0098-4FAC-B240-00AA00910026}">
+          <x14:cfRule type="cellIs" priority="10" operator="lessThan" id="{001100EF-00B9-481D-8AEA-00C500DB0049}">
             <xm:f>0</xm:f>
             <x14:dxf>
               <font>
@@ -5425,7 +5424,7 @@
           <xm:sqref>G2:G51</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="10" operator="lessThan" id="{008700F8-0038-43BC-B5E6-0044009B004A}">
+          <x14:cfRule type="cellIs" priority="10" operator="lessThan" id="{003000DB-0059-4520-9FCE-00FC009E0002}">
             <xm:f>0</xm:f>
             <x14:dxf>
               <font>
@@ -5442,7 +5441,7 @@
           <xm:sqref>H2 H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44 H45 H46 H47 H48 H49 H50 H51</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="9" operator="greaterThan" id="{0064007F-000F-4375-95B0-00A60011003B}">
+          <x14:cfRule type="cellIs" priority="9" operator="greaterThan" id="{00B300D8-006A-4120-8960-00BF008F00EF}">
             <xm:f>0</xm:f>
             <x14:dxf>
               <font>
@@ -5459,7 +5458,7 @@
           <xm:sqref>G2:G51</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="9" operator="greaterThan" id="{000500DB-002A-4E56-94F2-0038003700D9}">
+          <x14:cfRule type="cellIs" priority="9" operator="greaterThan" id="{0035009E-00B1-4A9F-9D61-008E003A00D6}">
             <xm:f>0</xm:f>
             <x14:dxf>
               <font>
@@ -5476,7 +5475,7 @@
           <xm:sqref>H2 H3 H4 H5 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20 H21 H22 H23 H24 H25 H26 H27 H28 H29 H30 H31 H32 H33 H34 H35 H36 H37 H38 H39 H40 H41 H42 H43 H44 H45 H46 H47 H48 H49 H50 H51</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="8" operator="greaterThanOrEqual" id="{00590076-006B-406C-9CC3-00270037009A}">
+          <x14:cfRule type="cellIs" priority="8" operator="greaterThanOrEqual" id="{0056009E-0089-4728-B97E-00C000DD00E3}">
             <xm:f>0.30</xm:f>
             <x14:dxf>
               <font>
@@ -5493,7 +5492,7 @@
           <xm:sqref>J2:J51</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="7" operator="lessThan" id="{007F00F0-004D-4F0C-8A0D-008A00F700E9}">
+          <x14:cfRule type="cellIs" priority="7" operator="lessThan" id="{00F800A9-0012-4AB4-A65B-009700D200D0}">
             <xm:f>0.30</xm:f>
             <x14:dxf>
               <font>
@@ -5510,7 +5509,7 @@
           <xm:sqref>J2:J51</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="6" operator="greaterThanOrEqual" id="{00CD0050-0074-4EE8-A106-006C00FD00A8}">
+          <x14:cfRule type="cellIs" priority="6" operator="greaterThanOrEqual" id="{0008004A-005C-4276-BF6E-0074009B0015}">
             <xm:f>1</xm:f>
             <x14:dxf>
               <font>
@@ -5527,7 +5526,7 @@
           <xm:sqref>K2:K51</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="5" operator="lessThan" id="{004C00A3-00DF-44A9-8404-009800230024}">
+          <x14:cfRule type="cellIs" priority="5" operator="lessThan" id="{008C00C9-0076-4899-B24B-006E00670035}">
             <xm:f>1</xm:f>
             <x14:dxf>
               <font>
@@ -5544,7 +5543,7 @@
           <xm:sqref>K2:K51</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="4" operator="greaterThanOrEqual" id="{008200BE-0053-4429-A0E3-00F4004F00DF}">
+          <x14:cfRule type="cellIs" priority="4" operator="greaterThanOrEqual" id="{00B3007C-001B-4E6B-A469-0021008600EC}">
             <xm:f>0.30</xm:f>
             <x14:dxf>
               <font>
@@ -5561,7 +5560,7 @@
           <xm:sqref>L2:L51</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" id="{005C005A-00DB-4DC2-AE1A-003C00F1007F}">
+          <x14:cfRule type="cellIs" priority="3" operator="greaterThanOrEqual" id="{0040008A-00BB-4F57-A864-00AC007500D1}">
             <xm:f>0.20</xm:f>
             <x14:dxf>
               <font>
@@ -5578,7 +5577,7 @@
           <xm:sqref>L2:L51</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="2" operator="greaterThanOrEqual" id="{001900D7-0093-46A1-A575-00E400DA001A}">
+          <x14:cfRule type="cellIs" priority="2" operator="greaterThanOrEqual" id="{008C0089-00B0-43A9-A493-00FE00B000DB}">
             <xm:f>0.20</xm:f>
             <x14:dxf>
               <font>
@@ -5595,7 +5594,7 @@
           <xm:sqref>L2:L51</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="1" operator="lessThan" id="{00AB001F-008C-4AEA-A106-00D5009A0077}">
+          <x14:cfRule type="cellIs" priority="1" operator="lessThan" id="{0067006C-00AD-482D-A4E4-001300A200F2}">
             <xm:f>0.20</xm:f>
             <x14:dxf>
               <font>

</xml_diff>